<commit_message>
enable fact sheet comparison
</commit_message>
<xml_diff>
--- a/data/EEA/Health_Impacts_Germany.xlsx
+++ b/data/EEA/Health_Impacts_Germany.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lochmannm\Documents\GitHub\END2DALY\data\EEA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1AF83AEC-E603-4F29-8D80-3D35F5EBD96F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D0778A0-FE24-4F4E-B36A-C7247F47B94A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-1980" windowWidth="29040" windowHeight="17520" xr2:uid="{20A32E53-1E3C-48CD-957F-84D49F6824DF}"/>
+    <workbookView xWindow="28680" yWindow="-4335" windowWidth="29040" windowHeight="15720" xr2:uid="{20A32E53-1E3C-48CD-957F-84D49F6824DF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1251" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1253" uniqueCount="110">
   <si>
     <t>Threshold</t>
   </si>
@@ -366,6 +366,9 @@
   </si>
   <si>
     <t>x_mort_yll</t>
+  </si>
+  <si>
+    <t>all</t>
   </si>
 </sst>
 </file>
@@ -834,6 +837,9 @@
       <c r="E2" s="1" t="s">
         <v>16</v>
       </c>
+      <c r="F2" t="s">
+        <v>109</v>
+      </c>
       <c r="G2">
         <v>6883100</v>
       </c>
@@ -886,6 +892,9 @@
       </c>
       <c r="E3" s="1" t="s">
         <v>17</v>
+      </c>
+      <c r="F3" t="s">
+        <v>109</v>
       </c>
       <c r="G3">
         <v>1239500</v>

</xml_diff>